<commit_message>
Clean repository and add final delivery reports
</commit_message>
<xml_diff>
--- a/iterations/accessories/thin_sources_2026-04-18/output/thin_sources_report.xlsx
+++ b/iterations/accessories/thin_sources_2026-04-18/output/thin_sources_report.xlsx
@@ -779,12 +779,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>thin_exact_card</t>
+          <t>download_failed:http_403</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">

</xml_diff>